<commit_message>
aded some new module per req
</commit_message>
<xml_diff>
--- a/Alt Tag Automation/Alt Report.xlsx
+++ b/Alt Tag Automation/Alt Report.xlsx
@@ -1,28 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28129"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\susmitha.kristam\PythonAutomationScriptGenentech\AltTags\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Excel VBA Automation\Alt Tag Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC0A49D-BE7D-4127-94C7-83198324B283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{701C1F4C-8212-4580-97C1-CFC444DF96C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="22320" windowHeight="13176" tabRatio="894" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Alt mismatch" sheetId="6" r:id="rId1"/>
-    <sheet name="ImageNotPresentOnSite" sheetId="5" r:id="rId2"/>
-    <sheet name="PASSING OUTPUT" sheetId="7" r:id="rId3"/>
-    <sheet name="GeneralScenarios" sheetId="1" r:id="rId4"/>
-    <sheet name="Scenario3" sheetId="2" r:id="rId5"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId6"/>
-    <sheet name="Scenario6" sheetId="4" r:id="rId7"/>
+    <sheet name="s" sheetId="7" r:id="rId1"/>
+    <sheet name="Alt mismatch" sheetId="9" r:id="rId2"/>
+    <sheet name="ImageNossOnSite" sheetId="5" r:id="rId3"/>
+    <sheet name="Alt mismssatch" sheetId="6" r:id="rId4"/>
+    <sheet name="PASSING OUTPUT" sheetId="10" r:id="rId5"/>
+    <sheet name="URL MATRIX ALT" sheetId="11" r:id="rId6"/>
+    <sheet name="GeneralScenarios" sheetId="1" r:id="rId7"/>
+    <sheet name="Sheet2" sheetId="12" r:id="rId8"/>
+    <sheet name="Scenario6" sheetId="4" r:id="rId9"/>
+    <sheet name="Scenario3" sheetId="2" r:id="rId10"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">GeneralScenarios!$A$1:$L$321</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">GeneralScenarios!$A$1:$L$321</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">ImageNossOnSite!$A$1:$G$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4258" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4324" uniqueCount="239">
   <si>
     <t>Website</t>
   </si>
@@ -1917,6 +1922,12 @@
   <si>
     <t>I was able to capture for this image name as it has only one scenario
 Imag is FAIL and Alt is PASS</t>
+  </si>
+  <si>
+    <t>$B$59</t>
+  </si>
+  <si>
+    <t>url</t>
   </si>
 </sst>
 </file>
@@ -2315,12 +2326,502 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F7BAF55-9E56-4BC6-9DB2-51FD880C4E3E}">
-  <sheetPr codeName="Sheet6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5EA0856-8906-4356-942E-F3DFF74F66AD}">
+  <sheetPr codeName="Sheet7"/>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="s">
+        <v>229</v>
+      </c>
+      <c r="E3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="73.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.77734375" customWidth="1"/>
+    <col min="4" max="4" width="28" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D6" t="s">
+        <v>142</v>
+      </c>
+      <c r="E6" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>142</v>
+      </c>
+      <c r="E7" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" t="s">
+        <v>140</v>
+      </c>
+      <c r="C8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D8" t="s">
+        <v>142</v>
+      </c>
+      <c r="E8" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" t="s">
+        <v>140</v>
+      </c>
+      <c r="C9" t="s">
+        <v>153</v>
+      </c>
+      <c r="D9" t="s">
+        <v>142</v>
+      </c>
+      <c r="E9" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B10" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" t="s">
+        <v>155</v>
+      </c>
+      <c r="D10" t="s">
+        <v>142</v>
+      </c>
+      <c r="E10" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D11" t="s">
+        <v>142</v>
+      </c>
+      <c r="E11" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12" t="s">
+        <v>148</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>142</v>
+      </c>
+      <c r="E12" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" t="s">
+        <v>148</v>
+      </c>
+      <c r="C13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" t="s">
+        <v>142</v>
+      </c>
+      <c r="E13" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B14" t="s">
+        <v>140</v>
+      </c>
+      <c r="C14" t="s">
+        <v>141</v>
+      </c>
+      <c r="D14" t="s">
+        <v>142</v>
+      </c>
+      <c r="E14" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B15" t="s">
+        <v>140</v>
+      </c>
+      <c r="C15" t="s">
+        <v>159</v>
+      </c>
+      <c r="D15" t="s">
+        <v>142</v>
+      </c>
+      <c r="E15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C16" t="s">
+        <v>98</v>
+      </c>
+      <c r="D16" t="s">
+        <v>142</v>
+      </c>
+      <c r="E16" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B17" t="s">
+        <v>148</v>
+      </c>
+      <c r="C17" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" t="s">
+        <v>142</v>
+      </c>
+      <c r="E17" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B18" t="s">
+        <v>140</v>
+      </c>
+      <c r="C18" t="s">
+        <v>141</v>
+      </c>
+      <c r="D18" t="s">
+        <v>142</v>
+      </c>
+      <c r="E18" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B19" t="s">
+        <v>148</v>
+      </c>
+      <c r="C19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" t="s">
+        <v>142</v>
+      </c>
+      <c r="E19" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B20" t="s">
+        <v>140</v>
+      </c>
+      <c r="C20" t="s">
+        <v>146</v>
+      </c>
+      <c r="D20" t="s">
+        <v>142</v>
+      </c>
+      <c r="E20" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" t="s">
+        <v>140</v>
+      </c>
+      <c r="C21" t="s">
+        <v>163</v>
+      </c>
+      <c r="D21" t="s">
+        <v>142</v>
+      </c>
+      <c r="E21" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B22" t="s">
+        <v>148</v>
+      </c>
+      <c r="C22" t="s">
+        <v>21</v>
+      </c>
+      <c r="D22" t="s">
+        <v>142</v>
+      </c>
+      <c r="E22" t="s">
+        <v>152</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="A7" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
+    <hyperlink ref="A8" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
+    <hyperlink ref="A9" r:id="rId8" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
+    <hyperlink ref="A10" r:id="rId9" xr:uid="{00000000-0004-0000-0100-000008000000}"/>
+    <hyperlink ref="A11" r:id="rId10" xr:uid="{00000000-0004-0000-0100-000009000000}"/>
+    <hyperlink ref="A12" r:id="rId11" xr:uid="{00000000-0004-0000-0100-00000A000000}"/>
+    <hyperlink ref="A13" r:id="rId12" xr:uid="{00000000-0004-0000-0100-00000B000000}"/>
+    <hyperlink ref="A14" r:id="rId13" xr:uid="{00000000-0004-0000-0100-00000C000000}"/>
+    <hyperlink ref="A15" r:id="rId14" xr:uid="{00000000-0004-0000-0100-00000D000000}"/>
+    <hyperlink ref="A16" r:id="rId15" xr:uid="{00000000-0004-0000-0100-00000E000000}"/>
+    <hyperlink ref="A17" r:id="rId16" xr:uid="{00000000-0004-0000-0100-00000F000000}"/>
+    <hyperlink ref="A18" r:id="rId17" xr:uid="{00000000-0004-0000-0100-000010000000}"/>
+    <hyperlink ref="A19" r:id="rId18" xr:uid="{00000000-0004-0000-0100-000011000000}"/>
+    <hyperlink ref="A20" r:id="rId19" xr:uid="{00000000-0004-0000-0100-000012000000}"/>
+    <hyperlink ref="A21" r:id="rId20" xr:uid="{00000000-0004-0000-0100-000013000000}"/>
+    <hyperlink ref="A22" r:id="rId21" xr:uid="{00000000-0004-0000-0100-000014000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr codeName="Sheet3"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0D24886-63ED-4ED0-82DC-E70DF59EC9C5}">
+  <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="44.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="53.77734375" customWidth="1"/>
+    <col min="4" max="4" width="23.5546875" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2436,10 +2937,10 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
         <v>14</v>
@@ -2448,10 +2949,10 @@
         <v>185</v>
       </c>
       <c r="E5" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="F5" t="s">
-        <v>117</v>
+        <v>11</v>
       </c>
       <c r="G5" t="e">
         <f>VLOOKUP(A5,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
@@ -2464,10 +2965,10 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
         <v>14</v>
@@ -2476,7 +2977,7 @@
         <v>185</v>
       </c>
       <c r="E6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F6" t="s">
         <v>117</v>
@@ -2492,10 +2993,10 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C7" t="s">
         <v>14</v>
@@ -2504,7 +3005,7 @@
         <v>185</v>
       </c>
       <c r="E7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F7" t="s">
         <v>117</v>
@@ -2520,10 +3021,10 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C8" t="s">
         <v>14</v>
@@ -2532,10 +3033,10 @@
         <v>185</v>
       </c>
       <c r="E8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F8" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="G8" t="e">
         <f>VLOOKUP(A8,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
@@ -2551,12 +3052,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64E4550D-9C58-45DA-92AC-04D0BDE7ECFD}">
-  <sheetPr codeName="Sheet5"/>
+  <sheetPr codeName="Sheet5" filterMode="1"/>
   <dimension ref="A1:I41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="65.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.44140625" customWidth="1"/>
     <col min="4" max="4" width="44.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.88671875" customWidth="1"/>
     <col min="7" max="7" width="37.33203125" bestFit="1" customWidth="1"/>
@@ -2606,15 +3109,15 @@
         <v>179</v>
       </c>
       <c r="F2" t="e">
-        <f>VLOOKUP(A2,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A2,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G2" t="e">
-        <f>VLOOKUP(B2,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B2,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="3" spans="1:9" s="4" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" s="4" customFormat="1" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>20</v>
       </c>
@@ -2631,18 +3134,18 @@
         <v>181</v>
       </c>
       <c r="F3" s="4" t="e">
-        <f>VLOOKUP(A3,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A3,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G3" s="4" t="e">
-        <f>VLOOKUP(B3,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B3,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="I3" s="8" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -2659,15 +3162,15 @@
         <v>183</v>
       </c>
       <c r="F4" t="e">
-        <f>VLOOKUP(A4,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A4,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G4" t="e">
-        <f>VLOOKUP(B4,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B4,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -2684,11 +3187,11 @@
         <v>184</v>
       </c>
       <c r="F5" t="e">
-        <f>VLOOKUP(A5,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A5,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G5" t="e">
-        <f>VLOOKUP(B5,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B5,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2709,11 +3212,11 @@
         <v>189</v>
       </c>
       <c r="F6" t="e">
-        <f>VLOOKUP(A6,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A6,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G6" t="e">
-        <f>VLOOKUP(B6,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B6,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2734,11 +3237,11 @@
         <v>190</v>
       </c>
       <c r="F7" t="e">
-        <f>VLOOKUP(A7,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A7,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G7" t="e">
-        <f>VLOOKUP(B7,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B7,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2759,11 +3262,11 @@
         <v>191</v>
       </c>
       <c r="F8" s="5" t="e">
-        <f>VLOOKUP(A8,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A8,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G8" s="5" t="str">
-        <f>VLOOKUP(B8,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B8,s!$B:$B,1,FALSE)</f>
         <v>Recurrence rates for stage II-IIIA NSCLC</v>
       </c>
       <c r="I8" s="6" t="s">
@@ -2787,11 +3290,11 @@
         <v>192</v>
       </c>
       <c r="F9" t="e">
-        <f>VLOOKUP(A9,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A9,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G9" t="e">
-        <f>VLOOKUP(B9,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B9,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2812,11 +3315,11 @@
         <v>193</v>
       </c>
       <c r="F10" t="e">
-        <f>VLOOKUP(A10,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A10,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G10" t="e">
-        <f>VLOOKUP(B10,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B10,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2837,11 +3340,11 @@
         <v>194</v>
       </c>
       <c r="F11" t="e">
-        <f>VLOOKUP(A11,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A11,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G11" t="e">
-        <f>VLOOKUP(B11,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B11,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2862,11 +3365,11 @@
         <v>195</v>
       </c>
       <c r="F12" t="e">
-        <f>VLOOKUP(A12,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A12,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G12" t="e">
-        <f>VLOOKUP(B12,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B12,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2887,11 +3390,11 @@
         <v>196</v>
       </c>
       <c r="F13" t="e">
-        <f>VLOOKUP(A13,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A13,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G13" t="e">
-        <f>VLOOKUP(B13,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B13,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2912,11 +3415,11 @@
         <v>197</v>
       </c>
       <c r="F14" t="e">
-        <f>VLOOKUP(A14,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A14,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G14" t="e">
-        <f>VLOOKUP(B14,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B14,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2937,11 +3440,11 @@
         <v>198</v>
       </c>
       <c r="F15" t="e">
-        <f>VLOOKUP(A15,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A15,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G15" t="e">
-        <f>VLOOKUP(B15,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B15,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2962,11 +3465,11 @@
         <v>199</v>
       </c>
       <c r="F16" t="e">
-        <f>VLOOKUP(A16,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A16,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G16" t="e">
-        <f>VLOOKUP(B16,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B16,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -2987,11 +3490,11 @@
         <v>200</v>
       </c>
       <c r="F17" t="e">
-        <f>VLOOKUP(A17,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A17,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G17" t="e">
-        <f>VLOOKUP(B17,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B17,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3012,11 +3515,11 @@
         <v>201</v>
       </c>
       <c r="F18" t="e">
-        <f>VLOOKUP(A18,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A18,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G18" t="e">
-        <f>VLOOKUP(B18,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B18,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3037,11 +3540,11 @@
         <v>202</v>
       </c>
       <c r="F19" t="e">
-        <f>VLOOKUP(A19,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A19,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G19" t="e">
-        <f>VLOOKUP(B19,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B19,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3062,11 +3565,11 @@
         <v>203</v>
       </c>
       <c r="F20" t="e">
-        <f>VLOOKUP(A20,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A20,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G20" t="e">
-        <f>VLOOKUP(B20,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B20,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3087,11 +3590,11 @@
         <v>204</v>
       </c>
       <c r="F21" t="e">
-        <f>VLOOKUP(A21,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A21,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G21" t="e">
-        <f>VLOOKUP(B21,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B21,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3112,11 +3615,11 @@
         <v>205</v>
       </c>
       <c r="F22" t="e">
-        <f>VLOOKUP(A22,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A22,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G22" t="e">
-        <f>VLOOKUP(B22,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B22,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3137,11 +3640,11 @@
         <v>206</v>
       </c>
       <c r="F23" t="e">
-        <f>VLOOKUP(A23,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A23,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G23" t="e">
-        <f>VLOOKUP(B23,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B23,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3162,11 +3665,11 @@
         <v>207</v>
       </c>
       <c r="F24" t="e">
-        <f>VLOOKUP(A24,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A24,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G24" t="e">
-        <f>VLOOKUP(B24,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B24,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3187,11 +3690,11 @@
         <v>208</v>
       </c>
       <c r="F25" t="e">
-        <f>VLOOKUP(A25,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A25,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G25" t="e">
-        <f>VLOOKUP(B25,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B25,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3212,11 +3715,11 @@
         <v>209</v>
       </c>
       <c r="F26" t="e">
-        <f>VLOOKUP(A26,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A26,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G26" t="e">
-        <f>VLOOKUP(B26,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B26,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3237,11 +3740,11 @@
         <v>210</v>
       </c>
       <c r="F27" t="e">
-        <f>VLOOKUP(A27,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A27,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G27" t="e">
-        <f>VLOOKUP(B27,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B27,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3262,11 +3765,11 @@
         <v>211</v>
       </c>
       <c r="F28" t="e">
-        <f>VLOOKUP(A28,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A28,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G28" t="e">
-        <f>VLOOKUP(B28,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B28,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3287,11 +3790,11 @@
         <v>212</v>
       </c>
       <c r="F29" t="e">
-        <f>VLOOKUP(A29,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A29,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G29" t="e">
-        <f>VLOOKUP(B29,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B29,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3312,11 +3815,11 @@
         <v>213</v>
       </c>
       <c r="F30" t="e">
-        <f>VLOOKUP(A30,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A30,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G30" t="e">
-        <f>VLOOKUP(B30,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B30,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3337,11 +3840,11 @@
         <v>214</v>
       </c>
       <c r="F31" t="e">
-        <f>VLOOKUP(A31,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A31,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G31" t="e">
-        <f>VLOOKUP(B31,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B31,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3362,11 +3865,11 @@
         <v>215</v>
       </c>
       <c r="F32" s="5" t="e">
-        <f>VLOOKUP(A32,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A32,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G32" s="5" t="e">
-        <f>VLOOKUP(B32,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B32,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="I32" s="6" t="s">
@@ -3390,11 +3893,11 @@
         <v>216</v>
       </c>
       <c r="F33" t="e">
-        <f>VLOOKUP(A33,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A33,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G33" t="e">
-        <f>VLOOKUP(B33,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B33,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3415,11 +3918,11 @@
         <v>217</v>
       </c>
       <c r="F34" t="e">
-        <f>VLOOKUP(A34,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A34,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G34" t="e">
-        <f>VLOOKUP(B34,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B34,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3440,11 +3943,11 @@
         <v>218</v>
       </c>
       <c r="F35" t="e">
-        <f>VLOOKUP(A35,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A35,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G35" t="e">
-        <f>VLOOKUP(B35,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B35,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3465,11 +3968,11 @@
         <v>219</v>
       </c>
       <c r="F36" t="e">
-        <f>VLOOKUP(A36,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A36,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G36" t="e">
-        <f>VLOOKUP(B36,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B36,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3490,11 +3993,11 @@
         <v>220</v>
       </c>
       <c r="F37" t="e">
-        <f>VLOOKUP(A37,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A37,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G37" t="e">
-        <f>VLOOKUP(B37,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B37,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3515,11 +4018,11 @@
         <v>221</v>
       </c>
       <c r="F38" t="e">
-        <f>VLOOKUP(A38,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A38,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G38" t="e">
-        <f>VLOOKUP(B38,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B38,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3540,11 +4043,11 @@
         <v>222</v>
       </c>
       <c r="F39" t="e">
-        <f>VLOOKUP(A39,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A39,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G39" t="e">
-        <f>VLOOKUP(B39,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B39,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3565,11 +4068,11 @@
         <v>223</v>
       </c>
       <c r="F40" t="e">
-        <f>VLOOKUP(A40,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A40,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G40" t="e">
-        <f>VLOOKUP(B40,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B40,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -3590,23 +4093,269 @@
         <v>224</v>
       </c>
       <c r="F41" t="e">
-        <f>VLOOKUP(A41,'PASSING OUTPUT'!$A:$A,1,FALSE)</f>
+        <f>VLOOKUP(A41,s!$A:$A,1,FALSE)</f>
         <v>#N/A</v>
       </c>
       <c r="G41" t="e">
-        <f>VLOOKUP(B41,'PASSING OUTPUT'!$B:$B,1,FALSE)</f>
+        <f>VLOOKUP(B41,s!$B:$B,1,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G41" xr:uid="{64E4550D-9C58-45DA-92AC-04D0BDE7ECFD}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="Image name and Alt tag not present on the Site"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5EA0856-8906-4356-942E-F3DFF74F66AD}">
-  <sheetPr codeName="Sheet7"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F7BAF55-9E56-4BC6-9DB2-51FD880C4E3E}">
+  <sheetPr codeName="Sheet6"/>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="39.21875" customWidth="1"/>
+    <col min="2" max="2" width="80.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="0" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="e">
+        <f>VLOOKUP(A2,s!$A:$A,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H2" t="e">
+        <f>VLOOKUP(B2,s!$B:$B,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E3" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="e">
+        <f>VLOOKUP(A3,s!$A:$A,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H3" t="e">
+        <f>VLOOKUP(B3,s!$B:$B,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>185</v>
+      </c>
+      <c r="E4" t="s">
+        <v>188</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="e">
+        <f>VLOOKUP(A4,s!$A:$A,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H4" t="e">
+        <f>VLOOKUP(B4,s!$B:$B,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>185</v>
+      </c>
+      <c r="E5" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G5" t="e">
+        <f>VLOOKUP(A5,s!$A:$A,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H5" t="e">
+        <f>VLOOKUP(B5,s!$B:$B,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>185</v>
+      </c>
+      <c r="E6" t="s">
+        <v>226</v>
+      </c>
+      <c r="F6" t="s">
+        <v>117</v>
+      </c>
+      <c r="G6" t="e">
+        <f>VLOOKUP(A6,s!$A:$A,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H6" t="e">
+        <f>VLOOKUP(B6,s!$B:$B,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>185</v>
+      </c>
+      <c r="E7" t="s">
+        <v>227</v>
+      </c>
+      <c r="F7" t="s">
+        <v>117</v>
+      </c>
+      <c r="G7" t="e">
+        <f>VLOOKUP(A7,s!$A:$A,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H7" t="e">
+        <f>VLOOKUP(B7,s!$B:$B,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
+        <v>185</v>
+      </c>
+      <c r="E8" t="s">
+        <v>228</v>
+      </c>
+      <c r="F8" t="s">
+        <v>129</v>
+      </c>
+      <c r="G8" t="e">
+        <f>VLOOKUP(A8,s!$A:$A,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H8" t="e">
+        <f>VLOOKUP(B8,s!$B:$B,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47613D89-ADF2-4364-A331-C97B91AEBCF2}">
+  <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -3666,13 +4415,35 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CF94D4E-BADA-4754-870E-E791031D66A4}">
+  <sheetPr codeName="Sheet8"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="60.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1" filterMode="1"/>
   <dimension ref="A1:L321"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="28.88671875" customWidth="1"/>
+    <col min="1" max="1" width="67.88671875" customWidth="1"/>
+    <col min="2" max="2" width="47.88671875" customWidth="1"/>
+    <col min="3" max="3" width="47.33203125" customWidth="1"/>
+    <col min="8" max="8" width="98.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
@@ -4283,7 +5054,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -6753,7 +7524,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>117</v>
       </c>
@@ -6791,7 +7562,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>117</v>
       </c>
@@ -6829,7 +7600,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>117</v>
       </c>
@@ -6867,7 +7638,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>117</v>
       </c>
@@ -6905,7 +7676,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>117</v>
       </c>
@@ -6943,7 +7714,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>117</v>
       </c>
@@ -7019,7 +7790,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>117</v>
       </c>
@@ -7095,7 +7866,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>117</v>
       </c>
@@ -7171,7 +7942,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>117</v>
       </c>
@@ -7285,7 +8056,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>117</v>
       </c>
@@ -7361,7 +8132,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>117</v>
       </c>
@@ -7399,7 +8170,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>117</v>
       </c>
@@ -7437,7 +8208,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="100" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>117</v>
       </c>
@@ -7475,7 +8246,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="101" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>117</v>
       </c>
@@ -7513,7 +8284,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="102" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>117</v>
       </c>
@@ -7551,7 +8322,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="103" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>117</v>
       </c>
@@ -7589,7 +8360,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>117</v>
       </c>
@@ -7627,7 +8398,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="105" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>117</v>
       </c>
@@ -7665,7 +8436,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="106" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>117</v>
       </c>
@@ -7703,7 +8474,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="107" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>117</v>
       </c>
@@ -7741,7 +8512,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="108" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>117</v>
       </c>
@@ -7779,7 +8550,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="109" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>117</v>
       </c>
@@ -7817,7 +8588,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="110" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>117</v>
       </c>
@@ -7855,7 +8626,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="111" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>117</v>
       </c>
@@ -7893,7 +8664,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="112" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>117</v>
       </c>
@@ -7931,7 +8702,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="113" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>117</v>
       </c>
@@ -7969,7 +8740,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>117</v>
       </c>
@@ -8007,7 +8778,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>117</v>
       </c>
@@ -8045,7 +8816,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>117</v>
       </c>
@@ -8083,7 +8854,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>117</v>
       </c>
@@ -8121,7 +8892,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>117</v>
       </c>
@@ -8159,7 +8930,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>117</v>
       </c>
@@ -8197,7 +8968,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>117</v>
       </c>
@@ -8235,7 +9006,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>117</v>
       </c>
@@ -8273,7 +9044,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>117</v>
       </c>
@@ -8311,7 +9082,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>117</v>
       </c>
@@ -8349,7 +9120,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>117</v>
       </c>
@@ -8425,7 +9196,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="126" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>117</v>
       </c>
@@ -8463,7 +9234,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="127" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>117</v>
       </c>
@@ -8501,7 +9272,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>117</v>
       </c>
@@ -8539,7 +9310,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="129" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>117</v>
       </c>
@@ -8577,7 +9348,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="130" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>117</v>
       </c>
@@ -8691,7 +9462,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="133" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>117</v>
       </c>
@@ -8729,7 +9500,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="134" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>117</v>
       </c>
@@ -8767,7 +9538,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="135" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>117</v>
       </c>
@@ -8805,7 +9576,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="136" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>117</v>
       </c>
@@ -8843,7 +9614,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="137" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>117</v>
       </c>
@@ -8881,7 +9652,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="138" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>117</v>
       </c>
@@ -8919,7 +9690,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="139" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>117</v>
       </c>
@@ -9109,7 +9880,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="144" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>117</v>
       </c>
@@ -9147,7 +9918,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="145" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>117</v>
       </c>
@@ -9185,7 +9956,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="146" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>117</v>
       </c>
@@ -9223,7 +9994,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="147" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>117</v>
       </c>
@@ -9261,7 +10032,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="148" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>117</v>
       </c>
@@ -9299,7 +10070,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="149" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>117</v>
       </c>
@@ -9337,7 +10108,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="150" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>117</v>
       </c>
@@ -9375,7 +10146,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="151" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>117</v>
       </c>
@@ -9413,7 +10184,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="152" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>117</v>
       </c>
@@ -9451,7 +10222,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="153" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>117</v>
       </c>
@@ -9489,7 +10260,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="154" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>117</v>
       </c>
@@ -9527,7 +10298,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="155" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>117</v>
       </c>
@@ -9565,7 +10336,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="156" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>117</v>
       </c>
@@ -9603,7 +10374,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="157" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>117</v>
       </c>
@@ -9641,7 +10412,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="158" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>117</v>
       </c>
@@ -9679,7 +10450,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="159" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>117</v>
       </c>
@@ -9717,7 +10488,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="160" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>117</v>
       </c>
@@ -9755,7 +10526,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="161" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>117</v>
       </c>
@@ -10363,7 +11134,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
         <v>124</v>
       </c>
@@ -13403,7 +14174,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" s="1" t="s">
         <v>129</v>
       </c>
@@ -15875,9 +16646,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L321" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
+    <filterColumn colId="0">
       <filters>
-        <filter val="tecentriq-ensclc-recurrence-rates-chart-mobile.svg"/>
+        <filter val="https://www.tecentriq-hcp.com/adjuvant-nsclc/about/how-tecentriq-works.html"/>
       </filters>
     </filterColumn>
     <filterColumn colId="4">
@@ -16212,417 +16983,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>136</v>
-      </c>
-      <c r="C1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D1" t="s">
-        <v>138</v>
-      </c>
-      <c r="E1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C2" t="s">
-        <v>141</v>
-      </c>
-      <c r="D2" t="s">
-        <v>142</v>
-      </c>
-      <c r="E2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C3" t="s">
-        <v>144</v>
-      </c>
-      <c r="D3" t="s">
-        <v>142</v>
-      </c>
-      <c r="E3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D4" t="s">
-        <v>142</v>
-      </c>
-      <c r="E4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s">
-        <v>148</v>
-      </c>
-      <c r="C5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" t="s">
-        <v>142</v>
-      </c>
-      <c r="E5" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" t="s">
-        <v>140</v>
-      </c>
-      <c r="C6" t="s">
-        <v>150</v>
-      </c>
-      <c r="D6" t="s">
-        <v>142</v>
-      </c>
-      <c r="E6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" t="s">
-        <v>148</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>142</v>
-      </c>
-      <c r="E7" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C8" t="s">
-        <v>141</v>
-      </c>
-      <c r="D8" t="s">
-        <v>142</v>
-      </c>
-      <c r="E8" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B9" t="s">
-        <v>140</v>
-      </c>
-      <c r="C9" t="s">
-        <v>153</v>
-      </c>
-      <c r="D9" t="s">
-        <v>142</v>
-      </c>
-      <c r="E9" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B10" t="s">
-        <v>140</v>
-      </c>
-      <c r="C10" t="s">
-        <v>155</v>
-      </c>
-      <c r="D10" t="s">
-        <v>142</v>
-      </c>
-      <c r="E10" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B11" t="s">
-        <v>140</v>
-      </c>
-      <c r="C11" t="s">
-        <v>157</v>
-      </c>
-      <c r="D11" t="s">
-        <v>142</v>
-      </c>
-      <c r="E11" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" t="s">
-        <v>142</v>
-      </c>
-      <c r="E12" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B13" t="s">
-        <v>148</v>
-      </c>
-      <c r="C13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" t="s">
-        <v>142</v>
-      </c>
-      <c r="E13" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B14" t="s">
-        <v>140</v>
-      </c>
-      <c r="C14" t="s">
-        <v>141</v>
-      </c>
-      <c r="D14" t="s">
-        <v>142</v>
-      </c>
-      <c r="E14" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B15" t="s">
-        <v>140</v>
-      </c>
-      <c r="C15" t="s">
-        <v>159</v>
-      </c>
-      <c r="D15" t="s">
-        <v>142</v>
-      </c>
-      <c r="E15" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B16" t="s">
-        <v>148</v>
-      </c>
-      <c r="C16" t="s">
-        <v>98</v>
-      </c>
-      <c r="D16" t="s">
-        <v>142</v>
-      </c>
-      <c r="E16" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B17" t="s">
-        <v>148</v>
-      </c>
-      <c r="C17" t="s">
-        <v>21</v>
-      </c>
-      <c r="D17" t="s">
-        <v>142</v>
-      </c>
-      <c r="E17" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B18" t="s">
-        <v>140</v>
-      </c>
-      <c r="C18" t="s">
-        <v>141</v>
-      </c>
-      <c r="D18" t="s">
-        <v>142</v>
-      </c>
-      <c r="E18" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B19" t="s">
-        <v>148</v>
-      </c>
-      <c r="C19" t="s">
-        <v>56</v>
-      </c>
-      <c r="D19" t="s">
-        <v>142</v>
-      </c>
-      <c r="E19" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B20" t="s">
-        <v>140</v>
-      </c>
-      <c r="C20" t="s">
-        <v>146</v>
-      </c>
-      <c r="D20" t="s">
-        <v>142</v>
-      </c>
-      <c r="E20" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B21" t="s">
-        <v>140</v>
-      </c>
-      <c r="C21" t="s">
-        <v>163</v>
-      </c>
-      <c r="D21" t="s">
-        <v>142</v>
-      </c>
-      <c r="E21" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B22" t="s">
-        <v>148</v>
-      </c>
-      <c r="C22" t="s">
-        <v>21</v>
-      </c>
-      <c r="D22" t="s">
-        <v>142</v>
-      </c>
-      <c r="E22" t="s">
-        <v>152</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="A4" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="A5" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
-    <hyperlink ref="A6" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
-    <hyperlink ref="A7" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
-    <hyperlink ref="A8" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
-    <hyperlink ref="A9" r:id="rId8" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
-    <hyperlink ref="A10" r:id="rId9" xr:uid="{00000000-0004-0000-0100-000008000000}"/>
-    <hyperlink ref="A11" r:id="rId10" xr:uid="{00000000-0004-0000-0100-000009000000}"/>
-    <hyperlink ref="A12" r:id="rId11" xr:uid="{00000000-0004-0000-0100-00000A000000}"/>
-    <hyperlink ref="A13" r:id="rId12" xr:uid="{00000000-0004-0000-0100-00000B000000}"/>
-    <hyperlink ref="A14" r:id="rId13" xr:uid="{00000000-0004-0000-0100-00000C000000}"/>
-    <hyperlink ref="A15" r:id="rId14" xr:uid="{00000000-0004-0000-0100-00000D000000}"/>
-    <hyperlink ref="A16" r:id="rId15" xr:uid="{00000000-0004-0000-0100-00000E000000}"/>
-    <hyperlink ref="A17" r:id="rId16" xr:uid="{00000000-0004-0000-0100-00000F000000}"/>
-    <hyperlink ref="A18" r:id="rId17" xr:uid="{00000000-0004-0000-0100-000010000000}"/>
-    <hyperlink ref="A19" r:id="rId18" xr:uid="{00000000-0004-0000-0100-000011000000}"/>
-    <hyperlink ref="A20" r:id="rId19" xr:uid="{00000000-0004-0000-0100-000012000000}"/>
-    <hyperlink ref="A21" r:id="rId20" xr:uid="{00000000-0004-0000-0100-000013000000}"/>
-    <hyperlink ref="A22" r:id="rId21" xr:uid="{00000000-0004-0000-0100-000014000000}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr codeName="Sheet3"/>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF49C61A-B50C-46D0-8487-20A72CA75C1E}">
+  <sheetPr codeName="Sheet11"/>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
@@ -16630,7 +16993,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:D5"/>

</xml_diff>